<commit_message>
Satın alma yolculuğu bölümü (site içi arama testi, sepet ve üyeliksiz ödeme akışı), GEO Promptları alt sayfası, bölüm içi veri seti butonları
- b_yolculuk.py: keşiften satış sonrasına adımlar, 38 aramalık site içi arama testi, sepet ve ödeme ekranları, önceliklendirilmiş dönüşüm fırsatları
- GEO: veri kaynakları tablosu (107 kelimelik gözlem, Search Console, 125 prompt), GEO Promptları sayfası (prompt oranları ve son yanıt metinleri)
- Üst bar: Pazaryeri Yorumları ve GEO Promptları butonları; ilgili alt başlıklardan alt sayfalara bağlantı

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Yöntem" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01 Kaynaklar'!$A$4:$H$1303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01 Kaynaklar'!$A$4:$H$1305</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02 Alan adı özeti'!$A$4:$E$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03 Yöntem'!$A$4:$A$23</definedName>
   </definedNames>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1303"/>
+  <dimension ref="A1:H1305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -507,7 +507,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VitrA e-ticaret büyüme fırsatları · kaynak siteler ve sayfalar (1299 satır, 77 alan adı)</t>
+          <t>VitrA e-ticaret büyüme fırsatları · kaynak siteler ve sayfalar (1301 satır, 77 alan adı)</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 25 Sonraki Adımlar</t>
+          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 04 SSG ve BM: Derin Talep İncelemesi · 05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 Organik Kanal Performansı · 23 Kanal Rolleri ve Etkileşim Modeli · 25 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 04 SSG ve BM: Derin Talep İncelemesi · 05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 Organik Kanal Performansı · 24 Kanal Rolleri ve Etkileşim Modeli · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 12 Yeni Kategori ve Segment Fırsatları · 25 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 12 Yeni Kategori ve Segment Fırsatları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 04 SSG ve BM: Derin Talep İncelemesi · 05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 Organik Kanal Performansı · 08 Google Arama Sonuçları ve AI Overview · 11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Rolleri ve Etkileşim Modeli · 25 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 04 SSG ve BM: Derin Talep İncelemesi · 05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 Organik Kanal Performansı · 08 Google Arama Sonuçları ve AI Overview · 11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 24 Kanal Rolleri ve Etkileşim Modeli · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>04 SSG ve BM: Derin Talep İncelemesi · 08 Google Arama Sonuçları ve AI Overview · 11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 25 Sonraki Adımlar</t>
+          <t>04 SSG ve BM: Derin Talep İncelemesi · 08 Google Arama Sonuçları ve AI Overview · 11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>04 SSG ve BM: Derin Talep İncelemesi · 11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Rolleri ve Etkileşim Modeli · 25 Sonraki Adımlar</t>
+          <t>04 SSG ve BM: Derin Talep İncelemesi · 11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 24 Kanal Rolleri ve Etkileşim Modeli · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 Organik Kanal Performansı · 07 Marka Aramaları ve Autocomplete · 08 Google Arama Sonuçları ve AI Overview · 09 YouTube: Montaj, Tamir ve Karar Videoları · 11 Katalog ve Talep Eşleşmesi · 13 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Rolleri ve Etkileşim Modeli · 25 Sonraki Adımlar</t>
+          <t>05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 Organik Kanal Performansı · 07 Marka Aramaları ve Autocomplete · 08 Google Arama Sonuçları ve AI Overview · 09 YouTube: Montaj, Tamir ve Karar Videoları · 11 Katalog ve Talep Eşleşmesi · 13 Set, Komple Banyo ve Ürün + Hizmet · 24 Kanal Rolleri ve Etkileşim Modeli · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>06 Organik Kanal Performansı · 13 Set, Komple Banyo ve Ürün + Hizmet · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>06 Organik Kanal Performansı · 13 Set, Komple Banyo ve Ürün + Hizmet · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>07 Marka Aramaları ve Autocomplete · 23 Kanal Rolleri ve Etkileşim Modeli · 25 Sonraki Adımlar</t>
+          <t>07 Marka Aramaları ve Autocomplete · 24 Kanal Rolleri ve Etkileşim Modeli · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>07 Marka Aramaları ve Autocomplete · 08 Google Arama Sonuçları ve AI Overview · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 23 Kanal Rolleri ve Etkileşim Modeli · 24 AI Arama ve GEO Fırsatları · 25 Sonraki Adımlar</t>
+          <t>07 Marka Aramaları ve Autocomplete · 08 Google Arama Sonuçları ve AI Overview · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 24 Kanal Rolleri ve Etkileşim Modeli · 25 AI Arama ve GEO Fırsatları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>API (DataForSEO SERP) · yapay zeka yanıt takibi (günlük ve haftalık koşu)</t>
+          <t>API (DataForSEO SERP) · yapay zeka yanıt takibi (tekrarlı koşu)</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>09 YouTube: Montaj, Tamir ve Karar Videoları · 24 AI Arama ve GEO Fırsatları · 25 Sonraki Adımlar</t>
+          <t>09 YouTube: Montaj, Tamir ve Karar Videoları · 25 AI Arama ve GEO Fırsatları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>09 YouTube: Montaj, Tamir ve Karar Videoları · 24 AI Arama ve GEO Fırsatları · 25 Sonraki Adımlar</t>
+          <t>09 YouTube: Montaj, Tamir ve Karar Videoları · 25 AI Arama ve GEO Fırsatları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -5461,7 +5461,7 @@
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>10 Şikayetvar: Satış Sonrası Deneyim · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 21 Kanal Politikaları ve Keşif Kanalları · 25 Sonraki Adımlar</t>
+          <t>10 Şikayetvar: Satış Sonrası Deneyim · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 21 Kanal Politikaları ve Keşif Kanalları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E119" s="6" t="inlineStr">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Rolleri ve Etkileşim Modeli · 25 Sonraki Adımlar</t>
+          <t>11 Katalog ve Talep Eşleşmesi · 12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 24 Kanal Rolleri ve Etkileşim Modeli · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E147" s="6" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E148" s="6" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E149" s="6" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E150" s="6" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E151" s="6" t="inlineStr">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E152" s="6" t="inlineStr">
@@ -6889,7 +6889,7 @@
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E153" s="6" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E155" s="6" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="D156" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E156" s="6" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E157" s="6" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="D158" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E158" s="6" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E159" s="6" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="D160" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E160" s="6" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E161" s="6" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E162" s="6" t="inlineStr">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E163" s="6" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="D164" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E164" s="6" t="inlineStr">
@@ -7393,7 +7393,7 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E165" s="6" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E166" s="6" t="inlineStr">
@@ -7477,7 +7477,7 @@
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E167" s="6" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E168" s="6" t="inlineStr">
@@ -7561,7 +7561,7 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E169" s="6" t="inlineStr">
@@ -7603,7 +7603,7 @@
       </c>
       <c r="D170" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E170" s="6" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="D172" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E172" s="6" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E173" s="6" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="D174" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E174" s="6" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E175" s="6" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="D176" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E176" s="6" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E177" s="6" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E178" s="6" t="inlineStr">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E179" s="6" t="inlineStr">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="D180" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E180" s="6" t="inlineStr">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 23 Kanal Rolleri ve Etkileşim Modeli</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 24 Kanal Rolleri ve Etkileşim Modeli</t>
         </is>
       </c>
       <c r="E181" s="6" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E182" s="6" t="inlineStr">
@@ -8149,7 +8149,7 @@
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 25 Sonraki Adımlar</t>
+          <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E183" s="6" t="inlineStr">
@@ -48133,7 +48133,7 @@
       </c>
       <c r="D1135" s="6" t="inlineStr">
         <is>
-          <t>20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 24 AI Arama ve GEO Fırsatları · 25 Sonraki Adımlar</t>
+          <t>20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 25 AI Arama ve GEO Fırsatları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E1135" s="6" t="inlineStr">
@@ -54544,111 +54544,111 @@
     <row r="1288" ht="30" customHeight="1">
       <c r="A1288" s="5" t="inlineStr">
         <is>
-          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
+          <t>https://www.vitra.com.tr/search?q=klozet+kapa%C4%9F%C4%B1</t>
         </is>
       </c>
       <c r="B1288" s="6" t="inlineStr">
         <is>
-          <t>duravit.com</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="C1288" s="6" t="inlineStr">
         <is>
-          <t>Duravit banyo planlayıcı (dijital deneyim aracı)</t>
+          <t>vitra.com.tr site içi arama testi (38 arama)</t>
         </is>
       </c>
       <c r="D1288" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>22 vitra.com.tr Satın Alma Yolculuğu: Site İçi Arama, Sepet ve Ödeme</t>
         </is>
       </c>
       <c r="E1288" s="6" t="inlineStr">
         <is>
-          <t>Banyo ölçüsüne göre ürün yerleştirme ve plan çıktısı</t>
+          <t>Sonuç sayısı, ilk 20 ürün kartı; 6 aramada sonuç yok; ilk kartlarda montaj hizmeti</t>
         </is>
       </c>
       <c r="F1288" s="7" t="inlineStr">
         <is>
-          <t>29.09.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="G1288" s="6" t="inlineStr">
         <is>
-          <t>tarayıcı</t>
+          <t>curl (herkese açık arama sayfası, istekler arası 2 sn)</t>
         </is>
       </c>
       <c r="H1288" s="7" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>D40</t>
         </is>
       </c>
     </row>
     <row r="1289" ht="30" customHeight="1">
       <c r="A1289" s="5" t="inlineStr">
         <is>
-          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
+          <t>https://www.vitra.com.tr/sepetim</t>
         </is>
       </c>
       <c r="B1289" s="6" t="inlineStr">
         <is>
-          <t>geberit.de</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="C1289" s="6" t="inlineStr">
         <is>
-          <t>Geberit AquaClean evde deneme programı (Almanya)</t>
+          <t>vitra.com.tr sepet, giriş ve üyeliksiz alışveriş ekranları</t>
         </is>
       </c>
       <c r="D1289" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>22 vitra.com.tr Satın Alma Yolculuğu: Site İçi Arama, Sepet ve Ödeme</t>
         </is>
       </c>
       <c r="E1289" s="6" t="inlineStr">
         <is>
-          <t>Dusch-WC'nin 4 hafta ücretsiz evde denenmesi, kurulum videosu ile</t>
+          <t>Sepeti Onayla → giriş paneli → e-posta ekranı → adres; montaj ve öneri karuselleri sepetin altında</t>
         </is>
       </c>
       <c r="F1289" s="7" t="inlineStr">
         <is>
-          <t>29.09.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="G1289" s="6" t="inlineStr">
         <is>
-          <t>tarayıcı</t>
+          <t>ekran görüntüsü (kullanıcı tarafından iletildi)</t>
         </is>
       </c>
       <c r="H1289" s="7" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>D41</t>
         </is>
       </c>
     </row>
     <row r="1290" ht="30" customHeight="1">
       <c r="A1290" s="5" t="inlineStr">
         <is>
-          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
+          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
         </is>
       </c>
       <c r="B1290" s="6" t="inlineStr">
         <is>
-          <t>grohe.com</t>
+          <t>duravit.com</t>
         </is>
       </c>
       <c r="C1290" s="6" t="inlineStr">
         <is>
-          <t>GROHE Spare Parts Finder (yedek parça bulucu örneği)</t>
+          <t>Duravit banyo planlayıcı (dijital deneyim aracı)</t>
         </is>
       </c>
       <c r="D1290" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E1290" s="6" t="inlineStr">
         <is>
-          <t>Patlatılmış çizim, parça numarası, montaj videosu; kamera ile ürün tanıma; üretimden kalkan ürünlerde 10 yıl parça güvencesi</t>
+          <t>Banyo ölçüsüne göre ürün yerleştirme ve plan çıktısı</t>
         </is>
       </c>
       <c r="F1290" s="7" t="inlineStr">
@@ -54663,34 +54663,34 @@
       </c>
       <c r="H1290" s="7" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>B10</t>
         </is>
       </c>
     </row>
     <row r="1291" ht="30" customHeight="1">
       <c r="A1291" s="5" t="inlineStr">
         <is>
-          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
+          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
         </is>
       </c>
       <c r="B1291" s="6" t="inlineStr">
         <is>
-          <t>hansgrohe-usa.com</t>
+          <t>geberit.de</t>
         </is>
       </c>
       <c r="C1291" s="6" t="inlineStr">
         <is>
-          <t>hansgrohe yedek parça arama (yedek parça bulucu örneği)</t>
+          <t>Geberit AquaClean evde deneme programı (Almanya)</t>
         </is>
       </c>
       <c r="D1291" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E1291" s="6" t="inlineStr">
         <is>
-          <t>Patlatılmış çizim, parça numarası ve montaj videosu ile yedek parça bulma; uyumluluk bilgisi</t>
+          <t>Dusch-WC'nin 4 hafta ücretsiz evde denenmesi, kurulum videosu ile</t>
         </is>
       </c>
       <c r="F1291" s="7" t="inlineStr">
@@ -54705,34 +54705,34 @@
       </c>
       <c r="H1291" s="7" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B13</t>
         </is>
       </c>
     </row>
     <row r="1292" ht="30" customHeight="1">
       <c r="A1292" s="5" t="inlineStr">
         <is>
-          <t>https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
+          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
         </is>
       </c>
       <c r="B1292" s="6" t="inlineStr">
         <is>
-          <t>victorianplumbing.co.uk</t>
+          <t>grohe.com</t>
         </is>
       </c>
       <c r="C1292" s="6" t="inlineStr">
         <is>
-          <t>Victorian Plumbing banyo finansmanı</t>
+          <t>GROHE Spare Parts Finder (yedek parça bulucu örneği)</t>
         </is>
       </c>
       <c r="D1292" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E1292" s="6" t="inlineStr">
         <is>
-          <t>250 GBP üzeri siparişte %0 faizli finansman; sepet tutarına bağlı finansman modeli</t>
+          <t>Patlatılmış çizim, parça numarası, montaj videosu; kamera ile ürün tanıma; üretimden kalkan ürünlerde 10 yıl parça güvencesi</t>
         </is>
       </c>
       <c r="F1292" s="7" t="inlineStr">
@@ -54747,34 +54747,34 @@
       </c>
       <c r="H1292" s="7" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>B12</t>
         </is>
       </c>
     </row>
     <row r="1293" ht="30" customHeight="1">
       <c r="A1293" s="5" t="inlineStr">
         <is>
-          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
+          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
         </is>
       </c>
       <c r="B1293" s="6" t="inlineStr">
         <is>
-          <t>villeroy-boch.co.uk</t>
+          <t>hansgrohe-usa.com</t>
         </is>
       </c>
       <c r="C1293" s="6" t="inlineStr">
         <is>
-          <t>Villeroy &amp; Boch 3D online banyo planlayıcı (dijital deneyim aracı)</t>
+          <t>hansgrohe yedek parça arama (yedek parça bulucu örneği)</t>
         </is>
       </c>
       <c r="D1293" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E1293" s="6" t="inlineStr">
         <is>
-          <t>Banyo ölçüsüne göre ürün yerleştirme, planın PDF olarak bayiye iletilmesi</t>
+          <t>Patlatılmış çizim, parça numarası ve montaj videosu ile yedek parça bulma; uyumluluk bilgisi</t>
         </is>
       </c>
       <c r="F1293" s="7" t="inlineStr">
@@ -54789,34 +54789,34 @@
       </c>
       <c r="H1293" s="7" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>B11</t>
         </is>
       </c>
     </row>
     <row r="1294" ht="30" customHeight="1">
       <c r="A1294" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/banyonu-tasarla</t>
+          <t>https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
         </is>
       </c>
       <c r="B1294" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr</t>
+          <t>victorianplumbing.co.uk</t>
         </is>
       </c>
       <c r="C1294" s="6" t="inlineStr">
         <is>
-          <t>VitrA V-Design (banyoyu tasarla) adresi: 3D planlayıcı durumu</t>
+          <t>Victorian Plumbing banyo finansmanı</t>
         </is>
       </c>
       <c r="D1294" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 25 Sonraki Adımlar</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E1294" s="6" t="inlineStr">
         <is>
-          <t>V-Design (2018) 750 banyo ve 300 karo ürünüyle tanıtılmıştı; adres bugün ana sayfaya yönleniyor</t>
+          <t>250 GBP üzeri siparişte %0 faizli finansman; sepet tutarına bağlı finansman modeli</t>
         </is>
       </c>
       <c r="F1294" s="7" t="inlineStr">
@@ -54831,182 +54831,182 @@
       </c>
       <c r="H1294" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B14</t>
         </is>
       </c>
     </row>
     <row r="1295" ht="30" customHeight="1">
       <c r="A1295" s="5" t="inlineStr">
         <is>
-          <t>https://chatgpt.com#ai-yanit</t>
+          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
         </is>
       </c>
       <c r="B1295" s="6" t="inlineStr">
         <is>
-          <t>chatgpt.com</t>
+          <t>villeroy-boch.co.uk</t>
         </is>
       </c>
       <c r="C1295" s="6" t="inlineStr">
         <is>
-          <t>ChatGPT yanıtları: 125 soruda VitrA ve rakip markaların adı geçme oranı, kaynak gösterilen alan adları</t>
+          <t>Villeroy &amp; Boch 3D online banyo planlayıcı (dijital deneyim aracı)</t>
         </is>
       </c>
       <c r="D1295" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E1295" s="6" t="inlineStr">
         <is>
-          <t>111 markasız ve 14 markalı soru; e-ticaret (20 soru) ve montaj (9 soru) grupları 28.09.2026'dan itibaren; 4 Eyl - 3 Eki 2026</t>
+          <t>Banyo ölçüsüne göre ürün yerleştirme, planın PDF olarak bayiye iletilmesi</t>
         </is>
       </c>
       <c r="F1295" s="7" t="inlineStr">
         <is>
-          <t>04.10.2026</t>
+          <t>29.09.2026</t>
         </is>
       </c>
       <c r="G1295" s="6" t="inlineStr">
         <is>
-          <t>yapay zeka yanıt takibi (günlük ve haftalık koşu)</t>
+          <t>tarayıcı</t>
         </is>
       </c>
       <c r="H1295" s="7" t="inlineStr">
         <is>
-          <t>D39</t>
+          <t>B9</t>
         </is>
       </c>
     </row>
     <row r="1296" ht="30" customHeight="1">
       <c r="A1296" s="5" t="inlineStr">
         <is>
-          <t>https://gemini.google.com#ai-yanit</t>
+          <t>https://www.vitra.com.tr/banyonu-tasarla</t>
         </is>
       </c>
       <c r="B1296" s="6" t="inlineStr">
         <is>
-          <t>google.com</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="C1296" s="6" t="inlineStr">
         <is>
-          <t>Gemini yanıtları: 125 soruda VitrA ve rakip markaların adı geçme oranı, kaynak gösterilen alan adları</t>
+          <t>VitrA V-Design (banyoyu tasarla) adresi: 3D planlayıcı durumu</t>
         </is>
       </c>
       <c r="D1296" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E1296" s="6" t="inlineStr">
         <is>
-          <t>111 markasız ve 14 markalı soru; e-ticaret (20 soru) ve montaj (9 soru) grupları 28.09.2026'dan itibaren; 4 Eyl - 3 Eki 2026</t>
+          <t>V-Design (2018) 750 banyo ve 300 karo ürünüyle tanıtılmıştı; adres bugün ana sayfaya yönleniyor</t>
         </is>
       </c>
       <c r="F1296" s="7" t="inlineStr">
         <is>
-          <t>04.10.2026</t>
+          <t>29.09.2026</t>
         </is>
       </c>
       <c r="G1296" s="6" t="inlineStr">
         <is>
-          <t>yapay zeka yanıt takibi (günlük ve haftalık koşu)</t>
+          <t>tarayıcı</t>
         </is>
       </c>
       <c r="H1296" s="7" t="inlineStr">
         <is>
-          <t>D39</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1297" ht="30" customHeight="1">
       <c r="A1297" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/llms.txt</t>
+          <t>https://chatgpt.com#ai-yanit</t>
         </is>
       </c>
       <c r="B1297" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr</t>
+          <t>chatgpt.com</t>
         </is>
       </c>
       <c r="C1297" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr llms.txt</t>
+          <t>ChatGPT yanıtları: 125 soruda VitrA ve rakip markaların adı geçme oranı, kaynak gösterilen alan adları</t>
         </is>
       </c>
       <c r="D1297" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="E1297" s="6" t="inlineStr">
         <is>
-          <t>Dosyadaki bölüm ve bağlantılar; destek ve rehber içeriğinin kapsamı</t>
+          <t>111 markasız ve 14 markalı soru; e-ticaret (20 soru) ve montaj (9 soru) grupları 28.09.2026'dan itibaren; 4 Eyl - 3 Eki 2026</t>
         </is>
       </c>
       <c r="F1297" s="7" t="inlineStr">
         <is>
-          <t>02.10.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="G1297" s="6" t="inlineStr">
         <is>
-          <t>web araştırması (sayfa okuma)</t>
+          <t>yapay zeka yanıt takibi (tekrarlı koşu)</t>
         </is>
       </c>
       <c r="H1297" s="7" t="inlineStr">
         <is>
-          <t>D35</t>
+          <t>D39</t>
         </is>
       </c>
     </row>
     <row r="1298" ht="30" customHeight="1">
       <c r="A1298" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/sitemaps/sitemap-ilham.xml</t>
+          <t>https://gemini.google.com#ai-yanit</t>
         </is>
       </c>
       <c r="B1298" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr</t>
+          <t>google.com</t>
         </is>
       </c>
       <c r="C1298" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr ilham site haritası</t>
+          <t>Gemini yanıtları: 125 soruda VitrA ve rakip markaların adı geçme oranı, kaynak gösterilen alan adları</t>
         </is>
       </c>
       <c r="D1298" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="E1298" s="6" t="inlineStr">
         <is>
-          <t>Rehber ve ilham sayfalarının listesi</t>
+          <t>111 markasız ve 14 markalı soru; e-ticaret (20 soru) ve montaj (9 soru) grupları 28.09.2026'dan itibaren; 4 Eyl - 3 Eki 2026</t>
         </is>
       </c>
       <c r="F1298" s="7" t="inlineStr">
         <is>
-          <t>02.10.2026</t>
+          <t>04.10.2026</t>
         </is>
       </c>
       <c r="G1298" s="6" t="inlineStr">
         <is>
-          <t>web araştırması (sayfa okuma)</t>
+          <t>yapay zeka yanıt takibi (tekrarlı koşu)</t>
         </is>
       </c>
       <c r="H1298" s="7" t="inlineStr">
         <is>
-          <t>D35</t>
+          <t>D39</t>
         </is>
       </c>
     </row>
     <row r="1299" ht="30" customHeight="1">
       <c r="A1299" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/sitemaps/sitemap-support.xml</t>
+          <t>https://www.vitra.com.tr/llms.txt</t>
         </is>
       </c>
       <c r="B1299" s="6" t="inlineStr">
@@ -55016,17 +55016,17 @@
       </c>
       <c r="C1299" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr destek site haritası</t>
+          <t>vitra.com.tr llms.txt</t>
         </is>
       </c>
       <c r="D1299" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="E1299" s="6" t="inlineStr">
         <is>
-          <t>Destek bölümündeki sayfa sayısı (5)</t>
+          <t>Dosyadaki bölüm ve bağlantılar; destek ve rehber içeriğinin kapsamı</t>
         </is>
       </c>
       <c r="F1299" s="7" t="inlineStr">
@@ -55048,27 +55048,27 @@
     <row r="1300" ht="30" customHeight="1">
       <c r="A1300" s="5" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q127325081</t>
+          <t>https://www.vitra.com.tr/sitemaps/sitemap-ilham.xml</t>
         </is>
       </c>
       <c r="B1300" s="6" t="inlineStr">
         <is>
-          <t>wikidata.org</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="C1300" s="6" t="inlineStr">
         <is>
-          <t>Wikidata ikinci VitrA kaydı</t>
+          <t>vitra.com.tr ilham site haritası</t>
         </is>
       </c>
       <c r="D1300" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="E1300" s="6" t="inlineStr">
         <is>
-          <t>Aynı marka için ayrı kayıt; alanlar ve bağlantılar</t>
+          <t>Rehber ve ilham sayfalarının listesi</t>
         </is>
       </c>
       <c r="F1300" s="7" t="inlineStr">
@@ -55083,34 +55083,34 @@
       </c>
       <c r="H1300" s="7" t="inlineStr">
         <is>
-          <t>D34</t>
+          <t>D35</t>
         </is>
       </c>
     </row>
     <row r="1301" ht="30" customHeight="1">
       <c r="A1301" s="5" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q7937213</t>
+          <t>https://www.vitra.com.tr/sitemaps/sitemap-support.xml</t>
         </is>
       </c>
       <c r="B1301" s="6" t="inlineStr">
         <is>
-          <t>wikidata.org</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="C1301" s="6" t="inlineStr">
         <is>
-          <t>Wikidata VitrA kaydı (marka ve entity tutarlılığı)</t>
+          <t>vitra.com.tr destek site haritası</t>
         </is>
       </c>
       <c r="D1301" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="E1301" s="6" t="inlineStr">
         <is>
-          <t>Kuruluş tarihi, üst kuruluş, web sitesi ve ürün grubu alanları</t>
+          <t>Destek bölümündeki sayfa sayısı (5)</t>
         </is>
       </c>
       <c r="F1301" s="7" t="inlineStr">
@@ -55125,34 +55125,34 @@
       </c>
       <c r="H1301" s="7" t="inlineStr">
         <is>
-          <t>D34</t>
+          <t>D35</t>
         </is>
       </c>
     </row>
     <row r="1302" ht="30" customHeight="1">
       <c r="A1302" s="5" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/VitrA_(sanitaryware)</t>
+          <t>https://www.wikidata.org/wiki/Q127325081</t>
         </is>
       </c>
       <c r="B1302" s="6" t="inlineStr">
         <is>
-          <t>wikipedia.org</t>
+          <t>wikidata.org</t>
         </is>
       </c>
       <c r="C1302" s="6" t="inlineStr">
         <is>
-          <t>İngilizce Wikipedia VitrA maddesi</t>
+          <t>Wikidata ikinci VitrA kaydı</t>
         </is>
       </c>
       <c r="D1302" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="E1302" s="6" t="inlineStr">
         <is>
-          <t>Kuruluş tarihi, üst kuruluş</t>
+          <t>Aynı marka için ayrı kayıt; alanlar ve bağlantılar</t>
         </is>
       </c>
       <c r="F1302" s="7" t="inlineStr">
@@ -55174,47 +55174,131 @@
     <row r="1303" ht="30" customHeight="1">
       <c r="A1303" s="5" t="inlineStr">
         <is>
+          <t>https://www.wikidata.org/wiki/Q7937213</t>
+        </is>
+      </c>
+      <c r="B1303" s="6" t="inlineStr">
+        <is>
+          <t>wikidata.org</t>
+        </is>
+      </c>
+      <c r="C1303" s="6" t="inlineStr">
+        <is>
+          <t>Wikidata VitrA kaydı (marka ve entity tutarlılığı)</t>
+        </is>
+      </c>
+      <c r="D1303" s="6" t="inlineStr">
+        <is>
+          <t>25 AI Arama ve GEO Fırsatları</t>
+        </is>
+      </c>
+      <c r="E1303" s="6" t="inlineStr">
+        <is>
+          <t>Kuruluş tarihi, üst kuruluş, web sitesi ve ürün grubu alanları</t>
+        </is>
+      </c>
+      <c r="F1303" s="7" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+      <c r="G1303" s="6" t="inlineStr">
+        <is>
+          <t>web araştırması (sayfa okuma)</t>
+        </is>
+      </c>
+      <c r="H1303" s="7" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304" ht="30" customHeight="1">
+      <c r="A1304" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/VitrA_(sanitaryware)</t>
+        </is>
+      </c>
+      <c r="B1304" s="6" t="inlineStr">
+        <is>
+          <t>wikipedia.org</t>
+        </is>
+      </c>
+      <c r="C1304" s="6" t="inlineStr">
+        <is>
+          <t>İngilizce Wikipedia VitrA maddesi</t>
+        </is>
+      </c>
+      <c r="D1304" s="6" t="inlineStr">
+        <is>
+          <t>25 AI Arama ve GEO Fırsatları</t>
+        </is>
+      </c>
+      <c r="E1304" s="6" t="inlineStr">
+        <is>
+          <t>Kuruluş tarihi, üst kuruluş</t>
+        </is>
+      </c>
+      <c r="F1304" s="7" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
+        </is>
+      </c>
+      <c r="G1304" s="6" t="inlineStr">
+        <is>
+          <t>web araştırması (sayfa okuma)</t>
+        </is>
+      </c>
+      <c r="H1304" s="7" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305" ht="30" customHeight="1">
+      <c r="A1305" s="5" t="inlineStr">
+        <is>
           <t>https://tr.wikipedia.org/wiki/VitrA</t>
         </is>
       </c>
-      <c r="B1303" s="6" t="inlineStr">
+      <c r="B1305" s="6" t="inlineStr">
         <is>
           <t>wikipedia.org</t>
         </is>
       </c>
-      <c r="C1303" s="6" t="inlineStr">
+      <c r="C1305" s="6" t="inlineStr">
         <is>
           <t>Türkçe Wikipedia VitrA maddesi</t>
         </is>
       </c>
-      <c r="D1303" s="6" t="inlineStr">
-        <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
-        </is>
-      </c>
-      <c r="E1303" s="6" t="inlineStr">
+      <c r="D1305" s="6" t="inlineStr">
+        <is>
+          <t>25 AI Arama ve GEO Fırsatları</t>
+        </is>
+      </c>
+      <c r="E1305" s="6" t="inlineStr">
         <is>
           <t>Kuruluş tarihi, Artema ilişkisi</t>
         </is>
       </c>
-      <c r="F1303" s="7" t="inlineStr">
+      <c r="F1305" s="7" t="inlineStr">
         <is>
           <t>02.10.2026</t>
         </is>
       </c>
-      <c r="G1303" s="6" t="inlineStr">
+      <c r="G1305" s="6" t="inlineStr">
         <is>
           <t>web araştırması (sayfa okuma)</t>
         </is>
       </c>
-      <c r="H1303" s="7" t="inlineStr">
+      <c r="H1305" s="7" t="inlineStr">
         <is>
           <t>D34</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H1303"/>
+  <autoFilter ref="A4:H1305"/>
   <mergeCells count="1">
     <mergeCell ref="A2:H2"/>
   </mergeCells>
@@ -56517,6 +56601,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1301" r:id="rId1296"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1302" r:id="rId1297"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1303" r:id="rId1298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1304" r:id="rId1299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1305" r:id="rId1300"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -56689,7 +56775,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>04 · 11 · 12 · 14 · 16 · 17 · 18 · 20 · 21 · 23 · 25</t>
+          <t>04 · 11 · 12 · 14 · 16 · 17 · 18 · 20 · 21 · 24 · 26</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -56714,7 +56800,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>10 · 13 · 14 · 16 · 17 · 18 · 20 · 21 · 22 · 25</t>
+          <t>10 · 13 · 14 · 16 · 17 · 18 · 20 · 21 · 23 · 26</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -56739,7 +56825,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>07 · 08 · 10 · 15 · 20 · 21 · 23 · 24 · 25</t>
+          <t>07 · 08 · 10 · 15 · 20 · 21 · 24 · 25 · 26</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -56753,103 +56839,103 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="43.5" customHeight="1">
+    <row r="9" ht="70.5" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>171</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>06 · 11 · 12 · 13 · 14 · 15 · 17 · 20 · 21 · 22 · 23 · 24 · 25 · 26</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>marka sitesi</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Yöntem: curl, tarayıcı, MCP (Ahrefs), API (Search Console), tarayıcı (Chrome, kullanıcı oturumu), tarayıcı (Playwright), curl (herkese açık arama sayfası, istekler arası 2 sn), ekran görüntüsü (kullanıcı tarafından iletildi), web araştırması (sayfa okuma); erişim 27.09.2026, 28.09.2026, 29.09.2026, 30.09.2026, 02.10.2026, 04.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="43.5" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>youtube.com</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B10" s="8" t="n">
         <v>167</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>09 YouTube: Montaj, Tamir ve Karar Videoları · 21 Kanal Politikaları ve Keşif Kanalları · 24 AI Arama ve GEO Fırsatları · 25 Sonraki Adımlar</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>09 YouTube: Montaj, Tamir ve Karar Videoları · 21 Kanal Politikaları ve Keşif Kanalları · 25 AI Arama ve GEO Fırsatları · 26 Sonraki Adımlar</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>sosyal</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Yöntem: API (DataForSEO YouTube), curl; erişim 28.09.2026, 29.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="57" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>cimri.com</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n">
-        <v>137</v>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>fiyat karşılaştırma</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Arama sayfası doğrulama katmanı nedeniyle açılamadı; kategori, marka ve ürün sayfaları Chrome ile okundu; 10 SKU eşleşmedi</t>
         </is>
       </c>
     </row>
     <row r="11" ht="57" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>cimri.com</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>137</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>fiyat karşılaştırma</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Arama sayfası doğrulama katmanı nedeniyle açılamadı; kategori, marka ve ürün sayfaları Chrome ile okundu; 10 SKU eşleşmedi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="57" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>akakce.com</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B12" s="8" t="n">
         <v>135</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 20 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>fiyat karşılaştırma</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Doğrudan erişim yaklaşık 15 istekten sonra doğrulama sayfası verdi (29.09.2026); 30.09.2026'da Chrome ile 24 ürün ve 12 kategori sayfası okundu</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="43.5" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>132</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>06 · 11 · 12 · 13 · 14 · 15 · 17 · 20 · 21 · 22 · 23 · 24 · 25</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>marka sitesi</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Yöntem: curl, tarayıcı, MCP (Ahrefs), API (Search Console), tarayıcı (Chrome, kullanıcı oturumu), tarayıcı (Playwright), web araştırması (sayfa okuma); erişim 27.09.2026, 28.09.2026, 29.09.2026, 30.09.2026, 02.10.2026</t>
         </is>
       </c>
     </row>
@@ -56864,7 +56950,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>03 · 04 · 05 · 06 · 07 · 08 · 09 · 11 · 12 · 13 · 20 · 21 · 23 · 24 · 25</t>
+          <t>03 · 04 · 05 · 06 · 07 · 08 · 09 · 11 · 12 · 13 · 20 · 21 · 24 · 25 · 26</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -56889,7 +56975,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>12 · 13 · 14 · 16 · 17 · 20 · 21 · 22</t>
+          <t>12 · 13 · 14 · 16 · 17 · 20 · 21 · 23</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -56939,7 +57025,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -56964,7 +57050,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 17 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -56989,7 +57075,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 25 Sonraki Adımlar</t>
+          <t>14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -57014,7 +57100,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>12 · 13 · 14 · 15 · 17 · 21 · 22</t>
+          <t>12 · 13 · 14 · 15 · 17 · 21 · 23</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -57064,7 +57150,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>03 · 04 · 05 · 06 · 07 · 08 · 09 · 10 · 11 · 12 · 13 · 15 · 20 · 21 · 23 · 24 · 25</t>
+          <t>03 · 04 · 05 · 06 · 07 · 08 · 09 · 10 · 11 · 12 · 13 · 15 · 20 · 21 · 24 · 25 · 26</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -57114,7 +57200,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -57139,7 +57225,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 25 Sonraki Adımlar</t>
+          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -57164,7 +57250,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 13 Set, Komple Banyo ve Ürün + Hizmet · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 15 Marka ve Uzman Sitelerde Kategori Trafiği · 21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -57339,7 +57425,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>21 Kanal Politikaları ve Keşif Kanalları · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>21 Kanal Politikaları ve Keşif Kanalları · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -57439,7 +57525,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -57464,7 +57550,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -57489,7 +57575,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -57514,7 +57600,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -57614,7 +57700,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -57678,7 +57764,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1">
+    <row r="46" ht="16.5" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>chatgpt.com</t>
@@ -57689,7 +57775,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>24 AI Arama ve GEO Fırsatları</t>
+          <t>25 AI Arama ve GEO Fırsatları</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -57699,7 +57785,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Yöntem: yapay zeka yanıt takibi (günlük ve haftalık koşu); erişim 04.10.2026</t>
+          <t>Yöntem: yapay zeka yanıt takibi (tekrarlı koşu); erişim 04.10.2026</t>
         </is>
       </c>
     </row>
@@ -57714,7 +57800,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -57839,7 +57925,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>12 Yeni Kategori ve Segment Fırsatları · 14 Rakip Görünürlüğü ve Kanal Ölçeği · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -57864,7 +57950,7 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -57889,7 +57975,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 12 Yeni Kategori ve Segment Fırsatları · 25 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 12 Yeni Kategori ve Segment Fırsatları · 26 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -57939,7 +58025,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -57989,7 +58075,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -58114,7 +58200,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>13 Set, Komple Banyo ve Ürün + Hizmet · 23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -58439,7 +58525,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>22 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>23 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -58657,7 +58743,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Kapsam: Bu döküm, rapor HTML'indeki 44 kaynakça girdisinin tüm adreslerini, rapordaki bağlantıları, alt ajan araştırmalarında (veri/ham/derin) okunan sayfaları ve API kaynaklarını içerir; 1299 satır, 77 alan adı. Toplu okunan sayfalar kalıp adres ve adet olarak tek satırdadır.</t>
+          <t>Kapsam: Bu döküm, rapor HTML'indeki 44 kaynakça girdisinin tüm adreslerini, rapordaki bağlantıları, alt ajan araştırmalarında (veri/ham/derin) okunan sayfaları ve API kaynaklarını içerir; 1301 satır, 77 alan adı. Toplu okunan sayfalar kalıp adres ve adet olarak tek satırdadır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aylık organik yatay ısı tabloları, kombo grafikler, çizgi/çubuk geçişi, tablo sütun seçimi, site geneli yapay zeka metrikleri
- Organik: 2025 Ocak-Mayıs (Search Console aylık dışa aktarımı) eklendi; Click, Gösterim, CTR, Ort. sıra için aylar sütunda yıllar satırda ısı tabloları; grafik sekmeleri: Click ve Gösterim (çizgi/çubuk), Click ve gösterim birlikte, 2026 için gösterim çubuk + tık çizgi + sıra kesikli çizgi
- Yeni kombo2 grafik (gruplu çubuk, çizgi, kesikli çizgi, üç eksen) ve cift (çizgi/çubuk geçişi)
- Tüm tablolarda Sütunlar düğmesi: sütunları göster/gizle, kopyalama yalnız görünen sütunları alır
- Yapay zeka bölümü: filtresiz dışa aktarımla site geneli gösterim ve pay (Mayıs %4,3 → Eylül %6,5), sayfa türüne göre, site genelinde en çok gösterilen sayfalar
- Ahrefs: pazaryeri ilk marka grubu, vitra.com.tr ve blog kuyrukları tamamlandı; marka analizi güncellendi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -1499,84 +1499,84 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="124.5" customHeight="1">
+    <row r="28" ht="97.5" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>https://ahrefs.com/site-explorer</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>ahrefs.com</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Organik rakipler, alan adı metrikleri, marka ve uzman sitelerin ve pazaryerlerinin kategori sayfası trafiği</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>06 Organik Kanal Performansı · 07 Google Yapay Zeka Özellikleri ve Organik Tık · 15 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Marka ve Uzman Sitelerde Kategori Trafiği · 17 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 25 Kanal Rolleri ve Etkileşim Modeli · 27 Sonraki Adımlar</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr'nin organik rakipleri (ilk 20) ve Batch Analysis (25 alan adı: DR, organik kelime, ilk 3, organik ve paid trafik; 27.09.2026); marka ve uzman siteler için top pages (26 hedef); pazaryeri ve yapı market için top pages ve organic keywords (10 site, Trendyol ve Hepsiburada 300'er kelime); Türkiye, 28.09.2026</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>27.09.2026 · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>33 · 36 · 35 · 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="124.5" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>https://www.vitra.com.tr</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>VitrA ana sayfa: şerit mesajları ve Banyo Asistanı akışı (taksit, kargo ve hizmet mesajı) | Rakip görünürlüğü ve kanal ölçeği: vitra.com.tr alan adı metrikleri (Ahrefs, Türkiye) | Marka ve uzman sitelerde kategori trafiği: vitra.com.tr tema × trafik matrisi (Ahrefs, Türkiye) | vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (ana sayfa)</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı · 14 Set, Komple Banyo ve Ürün + Hizmet · 15 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Marka ve Uzman Sitelerde Kategori Trafiği · 22 Kanal Politikaları ve Keşif Kanalları · 24 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Şeritte 'tüm ürünlerde vade farksız 6 ay taksit' ve 'tüm ürünlerde ücretsiz kargo'; Banyo Asistanı (Banyomu Yenilemek İstiyorum) 4 adımlı lead akışı: telefon, mağaza veya görüntülü görüşme seçimi, slot, WhatsApp teyidi; %40'a varan indirim, 9 taksit, ücretsiz mimari projelendirme | Batch Analysis: DR 66, 7.428 organik kelime, ilk 3'te 4.127 kelime, 330.499 organik ve 50.286 paid trafik (Ahrefs tahmini, 27.09.2026) | Ahrefs site toplamı: DR 66, 7.428 organik kelime, 330.499 aylık organik trafik; top pages: 138 sayfa 40'tan fazla temaya eşlendi (28.09.2026) | 1 Eki 2025 - 30 Eyl 2026: 134.587 tıklama, 4.500.313 gösterim, ortalama sıra 10</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>27.09.2026 · 28.09.2026 · 29.09.2026</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>11 · 33 · 22 · 35 · 47</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vitra.com.tr/c-banyo-dolaplari</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-banyo-dolaplari)</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>06 Organik Kanal Performansı</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 24.731 tıklama, 721.659 gösterim, ortalama sıra 6</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-banyo-karo-seramikleri</t>
+          <t>https://www.vitra.com.tr/c-banyo-dolaplari</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-banyo-karo-seramikleri)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-banyo-dolaplari)</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 32.464 tıklama, 1.193.310 gösterim, ortalama sıra 6</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 24.731 tıklama, 721.659 gösterim, ortalama sıra 6</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -1613,7 +1613,7 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-banyo-mobilyalari</t>
+          <t>https://www.vitra.com.tr/c-banyo-karo-seramikleri</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-banyo-mobilyalari)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-banyo-karo-seramikleri)</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 39.036 tıklama, 1.297.491 gösterim, ortalama sıra 5,5</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 32.464 tıklama, 1.193.310 gösterim, ortalama sıra 6</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -1650,7 +1650,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-dus-setleri</t>
+          <t>https://www.vitra.com.tr/c-banyo-mobilyalari</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-dus-setleri)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-banyo-mobilyalari)</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 18.435 tıklama, 647.203 gösterim, ortalama sıra 5,6</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 39.036 tıklama, 1.297.491 gösterim, ortalama sıra 5,5</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -1687,7 +1687,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-dus-tekneleri</t>
+          <t>https://www.vitra.com.tr/c-dus-setleri</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-dus-tekneleri)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-dus-setleri)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 18.923 tıklama, 432.258 gösterim, ortalama sıra 5,1</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 18.435 tıklama, 647.203 gösterim, ortalama sıra 5,6</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -1724,7 +1724,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-dusakabin</t>
+          <t>https://www.vitra.com.tr/c-dus-tekneleri</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-dusakabin)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-dus-tekneleri)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 47.218 tıklama, 1.578.979 gösterim, ortalama sıra 6,6</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 18.923 tıklama, 432.258 gösterim, ortalama sıra 5,1</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-ev-ici-zemin-karo-seramikleri</t>
+          <t>https://www.vitra.com.tr/c-dusakabin</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-ev-ici-zemin-karo-seramikleri)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-dusakabin)</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 19.416 tıklama, 878.622 gösterim, ortalama sıra 6,4</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 47.218 tıklama, 1.578.979 gösterim, ortalama sıra 6,6</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -1798,7 +1798,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-eviye-bataryalari</t>
+          <t>https://www.vitra.com.tr/c-ev-ici-zemin-karo-seramikleri</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-eviye-bataryalari)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-ev-ici-zemin-karo-seramikleri)</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 27.192 tıklama, 874.023 gösterim, ortalama sıra 5,5</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 19.416 tıklama, 878.622 gösterim, ortalama sıra 6,4</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
@@ -1835,7 +1835,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-gomme-rezervuarlar</t>
+          <t>https://www.vitra.com.tr/c-eviye-bataryalari</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-gomme-rezervuarlar)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-eviye-bataryalari)</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 24.686 tıklama, 709.966 gösterim, ortalama sıra 4,9</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 27.192 tıklama, 874.023 gösterim, ortalama sıra 5,5</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -1872,7 +1872,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-karo-seramik-urunleri</t>
+          <t>https://www.vitra.com.tr/c-gomme-rezervuarlar</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-karo-seramik-urunleri)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-gomme-rezervuarlar)</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 29.900 tıklama, 1.032.767 gösterim, ortalama sıra 6,3</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 24.686 tıklama, 709.966 gösterim, ortalama sıra 4,9</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -1909,7 +1909,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-klozetler</t>
+          <t>https://www.vitra.com.tr/c-karo-seramik-urunleri</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-klozetler)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-karo-seramik-urunleri)</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 60.921 tıklama, 2.302.714 gösterim, ortalama sıra 5,2</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 29.900 tıklama, 1.032.767 gösterim, ortalama sıra 6,3</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-lavabo-dolaplari</t>
+          <t>https://www.vitra.com.tr/c-klozetler</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-lavabo-dolaplari)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-klozetler)</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 21.562 tıklama, 740.877 gösterim, ortalama sıra 5,9</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 60.921 tıklama, 2.302.714 gösterim, ortalama sıra 5,2</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
@@ -1983,101 +1983,101 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
+          <t>https://www.vitra.com.tr/c-lavabo-dolaplari</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-lavabo-dolaplari)</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>06 Organik Kanal Performansı</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>1 Eki 2025 - 30 Eyl 2026: 21.562 tıklama, 740.877 gösterim, ortalama sıra 5,9</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
           <t>https://www.vitra.com.tr/c-lavabolar</t>
         </is>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/c-lavabolar)</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 45.640 tıklama, 1.777.097 gösterim, ortalama sıra 6,6</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="43.5" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43" ht="43.5" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/ahsap-gorunumlu-seramik-modelleri/</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/ahsap-gorunumlu-seramik-modelleri)</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 5.839 tıklama, 183.660 gösterim, ortalama sıra 6</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/banyo-temizligi-nasil-yapilir/</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/banyo-temizligi-nasil-yapilir)</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>06 Organik Kanal Performansı</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 1.618 tıklama, 239.581 gösterim, ortalama sıra 5,3</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -2094,7 +2094,7 @@
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/bide-nedir/</t>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/banyo-temizligi-nasil-yapilir/</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/bide-nedir)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/banyo-temizligi-nasil-yapilir)</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 3.226 tıklama, 386.711 gösterim, ortalama sıra 5</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 1.618 tıklama, 239.581 gösterim, ortalama sıra 5,3</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
@@ -2131,212 +2131,212 @@
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/bide-nedir/</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/bide-nedir)</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>06 Organik Kanal Performansı</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>1 Eki 2025 - 30 Eyl 2026: 3.226 tıklama, 386.711 gösterim, ortalama sıra 5</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/dusakabin-montaji-nasil-yapilir/</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/dusakabin-montaji-nasil-yapilir)</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 2.236 tıklama, 192.047 gösterim, ortalama sıra 5,3</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="43.5" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47" ht="43.5" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/dusakabin-temizligi-nasil-yapilir/</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/dusakabin-temizligi-nasil-yapilir)</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 8.681 tıklama, 564.677 gösterim, ortalama sıra 4</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/en-kullanisli-evye-hangisi/</t>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/en-kullanisli-evye-hangisi)</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 12.879 tıklama, 621.735 gösterim, ortalama sıra 7</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G48" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="43.5" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49" ht="43.5" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/gomme-rezervuar-montaji-nasil-yapilir/</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/gomme-rezervuar-montaji-nasil-yapilir)</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 2.535 tıklama, 298.519 gösterim, ortalama sıra 6,2</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G49" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/gomme-rezervuar-tamiri/</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/gomme-rezervuar-tamiri)</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 6.752 tıklama, 623.040 gösterim, ortalama sıra 5,7</t>
-        </is>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="43.5" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/kanalsiz-klozet-nedir-ve-nasil-calisir/</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/kanalsiz-klozet-nedir-ve-nasil-calisir)</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>06 Organik Kanal Performansı</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 1.821 tıklama, 83.454 gösterim, ortalama sıra 4,5</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
@@ -2353,7 +2353,7 @@
     <row r="51" ht="43.5" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/klozet-kapagi-montaji-nasil-yapilir/</t>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/kanalsiz-klozet-nedir-ve-nasil-calisir/</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/klozet-kapagi-montaji-nasil-yapilir)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/kanalsiz-klozet-nedir-ve-nasil-calisir)</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 2.468 tıklama, 351.426 gösterim, ortalama sıra 5,8</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 1.821 tıklama, 83.454 gösterim, ortalama sıra 4,5</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <row r="52" ht="43.5" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/klozet-secim-rehberi-ve-tavsiyeler/</t>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/klozet-kapagi-montaji-nasil-yapilir/</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/klozet-secim-rehberi-ve-tavsiyeler)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/klozet-kapagi-montaji-nasil-yapilir)</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 3.472 tıklama, 275.927 gösterim, ortalama sıra 5,5</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 2.468 tıklama, 351.426 gösterim, ortalama sıra 5,8</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -2427,7 +2427,7 @@
     <row r="53" ht="43.5" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/kucuk-banyolar-icin-karo-secimi-nasil-olmali/</t>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/klozet-secim-rehberi-ve-tavsiyeler/</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/kucuk-banyolar-icin-karo-secimi-nasil-olmali)</t>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/klozet-secim-rehberi-ve-tavsiyeler)</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 1.731 tıklama, 104.802 gösterim, ortalama sıra 6,6</t>
+          <t>1 Eki 2025 - 30 Eyl 2026: 3.472 tıklama, 275.927 gösterim, ortalama sıra 5,5</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -2464,64 +2464,64 @@
     <row r="54" ht="43.5" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/kucuk-banyolar-icin-karo-secimi-nasil-olmali/</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/kucuk-banyolar-icin-karo-secimi-nasil-olmali)</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>06 Organik Kanal Performansı</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>1 Eki 2025 - 30 Eyl 2026: 1.731 tıklama, 104.802 gösterim, ortalama sıra 6,6</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="43.5" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/lavabo-secim-rehberi-ve-tavsiyeler/</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/lavabo-secim-rehberi-ve-tavsiyeler)</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 1.467 tıklama, 167.001 gösterim, ortalama sıra 6,6</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>28.09.2026</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vitra.com.tr/ilham-veren-fikirler/mutfak-dekorasyonu-nasil-yapilir/</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/mutfak-dekorasyonu-nasil-yapilir)</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>06 Organik Kanal Performansı</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>1 Eki 2025 - 30 Eyl 2026: 2.865 tıklama, 466.233 gösterim, ortalama sıra 2,5</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2538,111 +2538,111 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
+          <t>https://www.vitra.com.tr/ilham-veren-fikirler/mutfak-dekorasyonu-nasil-yapilir/</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/mutfak-dekorasyonu-nasil-yapilir)</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>06 Organik Kanal Performansı</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>1 Eki 2025 - 30 Eyl 2026: 2.865 tıklama, 466.233 gösterim, ortalama sıra 2,5</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>28.09.2026</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
           <t>https://www.vitra.com.tr/ilham-veren-fikirler/vitrifiye-urun-gruplari-nelerdir/</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/vitrifiye-urun-gruplari-nelerdir)</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>1 Eki 2025 - 30 Eyl 2026: 1.617 tıklama, 118.742 gösterim, ortalama sıra 5,1</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G57" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="43.5" customHeight="1">
-      <c r="A57" s="5" t="inlineStr">
+    <row r="58" ht="43.5" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/servisler-ve-satis-noktalari</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>VitrA resmi satış ve servis noktası bulucusu | vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (/servisler-ve-satis-noktalari)</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>06 Organik Kanal Performansı · 22 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>161 satış noktası ve 76 servis noktası (toplam 237); Google Maps profilleriyle karşılaştırma için resmi sayı | 1 Eki 2025 - 30 Eyl 2026: 25.760 tıklama, 1.300.640 gösterim, ortalama sıra 5,1</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>28.09.2026 · 29.09.2026</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>11 · 47</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="84" customHeight="1">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>https://ahrefs.com/site-explorer</t>
-        </is>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>ahrefs.com</t>
-        </is>
-      </c>
-      <c r="C58" s="6" t="inlineStr">
-        <is>
-          <t>Organik rakipler, alan adı metrikleri, marka ve uzman sitelerin ve pazaryerlerinin kategori sayfası trafiği</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>07 Google Yapay Zeka Özellikleri ve Organik Tık · 15 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Marka ve Uzman Sitelerde Kategori Trafiği · 17 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 25 Kanal Rolleri ve Etkileşim Modeli · 27 Sonraki Adımlar</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>vitra.com.tr'nin organik rakipleri (ilk 20) ve Batch Analysis (25 alan adı: DR, organik kelime, ilk 3, organik ve paid trafik; 27.09.2026); marka ve uzman siteler için top pages (26 hedef); pazaryeri ve yapı market için top pages ve organic keywords (10 site, Trendyol ve Hepsiburada 300'er kelime); Türkiye, 28.09.2026</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>27.09.2026 · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>33 · 36 · 35 · 12</t>
         </is>
       </c>
     </row>
@@ -50776,7 +50776,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="57" customHeight="1">
+    <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>ahrefs.com</t>
@@ -50787,7 +50787,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>07 Google Yapay Zeka Özellikleri ve Organik Tık · 15 Rakip Görünürlüğü ve Kanal Ölçeği · 16 Marka ve Uzman Sitelerde Kategori Trafiği · 17 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 25 Kanal Rolleri ve Etkileşim Modeli · 27 Sonraki Adımlar</t>
+          <t>06 · 07 · 15 · 16 · 17 · 25 · 27</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">

</xml_diff>

<commit_message>
GA4: site içi arama örneklenmemiş Mayıs-Eylül dışa aktarımlarına, servis düğmesi tıklaması yıllı veriye taşındı; anahtar olay sütunları çıkarıldı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -52471,7 +52471,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="57" customHeight="1">
+    <row r="8" ht="70.5" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Google Analytics 4</t>
@@ -52479,7 +52479,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr mülkü, VitrA ekibi dışa aktarımı (05.10.2026) · genel bakış Oca 2025 - Eyl 2026 · kanal Oca - Eyl 2025 ve 2026 · site içi arama 1 Nis - 5 Eki 2026 · ödeme, teslimat, talep olayları, sayfa ve promosyon 1 Eyl 2025 - 30 Eyl 2026</t>
+          <t>vitra.com.tr mülkü, VitrA ekibi dışa aktarımı (05.10.2026) · genel bakış Oca 2025 - Eyl 2026 · kanal Oca - Eyl 2025 ve 2026 · site içi arama 1 May - 30 Eyl 2026 · ödeme, teslimat, servis düğmesi tıklaması, sayfa ve promosyon 1 Eyl 2025 - 30 Eyl 2026 · giriş sayfası Oca 2025 - 5 Eki 2026</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -52489,7 +52489,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Site içi arama keşif raporu örneklenmiştir; landing page dışa aktarımı süzgeç belirsizliği nedeniyle kullanılmamıştır</t>
+          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) sütunları tüm olayları kapsadığından kullanılmamıştır</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GA4: satın alma hunisi, yeni ve geri dönen kullanıcılar, ürün ve kategori performansı, blog oturumlarında ürüne geçiş
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -52471,7 +52471,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="70.5" customHeight="1">
+    <row r="8" ht="97.5" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Google Analytics 4</t>
@@ -52489,7 +52489,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır</t>
+          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) bazı aylarda geçersiz değer taşıdığından kullanılmamış; ürün geliri genel bakıştaki gelirden farklı hesaplandığı için pay olarak verilmiştir</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GA4: ödeme, teslimat ve promosyon son 12 ay; sepete ekleme oranı (hatalı kodlar hariç); blog oturumu kanal dağılımı; _ga bulgusu, kullanıcı düzeyi kırılım çıkarıldı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -52471,7 +52471,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="97.5" customHeight="1">
+    <row r="8" ht="138" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Google Analytics 4</t>
@@ -52479,7 +52479,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr mülkü, VitrA ekibi dışa aktarımı (05.10.2026) · genel bakış Oca 2025 - Eyl 2026 · kanal Oca - Eyl 2025 ve 2026 · site içi arama 1 May - 30 Eyl 2026 · ödeme, teslimat, servis düğmesi tıklaması, sayfa ve promosyon 1 Eyl 2025 - 30 Eyl 2026 · giriş sayfası Oca 2025 - 5 Eki 2026</t>
+          <t>vitra.com.tr mülkü, VitrA ekibi dışa aktarımı (05.10.2026) · genel bakış Oca 2025 - Eyl 2026 · kanal Oca - Eyl 2025 ve 2026 · site içi arama 1 May - 30 Eyl 2026 · ödeme, teslimat, servis düğmesi ve promosyon 1 Eki 2025 - 30 Eyl 2026 · blog ve koleksiyon sayfaları 1 Ara 2025 - 30 Eyl 2026 · giriş sayfası Oca 2025 - 5 Eki 2026 · huni ve ürün Oca 2025 - Eyl 2026</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -52489,7 +52489,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) bazı aylarda geçersiz değer taşıdığından kullanılmamış; ürün geliri genel bakıştaki gelirden farklı hesaplandığı için pay olarak verilmiştir</t>
+          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün geliri genel bakıştaki gelirden farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında oturum ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GA4: sipariş onay sayfasında yeni oturumun yönlendireni (iyzico) ve satın almanın kaynak / ortamı; grafik değer etiketlerinde çakışma önleme; blog Click + Gösterim sekmesi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -52471,7 +52471,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="138" customHeight="1">
+    <row r="8" ht="165" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Google Analytics 4</t>
@@ -52479,7 +52479,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>vitra.com.tr mülkü, VitrA ekibi dışa aktarımı (05.10.2026) · genel bakış Oca 2025 - Eyl 2026 · kanal Oca - Eyl 2025 ve 2026 · site içi arama 1 May - 30 Eyl 2026 · ödeme, teslimat, servis düğmesi ve promosyon 1 Eki 2025 - 30 Eyl 2026 · blog ve koleksiyon sayfaları 1 Ara 2025 - 30 Eyl 2026 · giriş sayfası Oca 2025 - 5 Eki 2026 · huni ve ürün Oca 2025 - Eyl 2026</t>
+          <t>vitra.com.tr mülkü, VitrA ekibi dışa aktarımı (05.10.2026) · genel bakış Oca 2025 - Eyl 2026 · kanal Oca - Eyl 2025 ve 2026 · site içi arama 1 May - 30 Eyl 2026 · ödeme, teslimat, servis düğmesi ve promosyon 1 Eki 2025 - 30 Eyl 2026 · blog ve koleksiyon sayfaları 1 Ara 2025 - 30 Eyl 2026 · giriş sayfası Oca 2025 - 5 Eki 2026 · sipariş onay sayfası 1 Eki 2025 - 30 Eyl 2026 · huni ve ürün Oca 2025 - Eyl 2026</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -52489,7 +52489,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün geliri genel bakıştaki gelirden farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında oturum ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir</t>
+          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün geliri genel bakıştaki gelirden farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında oturum ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir. Sipariş onay sayfası keşiflerinde (1 Eki 2025 - 30 Eyl 2026) bazı aylar örneklendiği için yalnız paylar kullanılmış; satın almanın kaynak / ortamı GA4 atama modeline göre, oturum kanalı ise oturum kanal grubuna göre verilmiştir</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablolara ısı haritası düğmesi (mevcut ısı tabloları açık, diğerleri kapalı; aynı metrik aynı renk); metrik adları rapor genelinde İngilizce (session, impression, click, revenue, search volume, view, visit, traffic, avg. position, AOV, purchase)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Tık · 08 GA4 - Site ve E-Ticaret Performansı · 09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 11 YouTube: Montaj, Tamir ve Karar Videoları · 13 Katalog ve Talep Eşleşmesi · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 08 GA4 - Site ve E-Ticaret Performansı · 09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 11 YouTube: Montaj, Tamir ve Karar Videoları · 13 Katalog ve Talep Eşleşmesi · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Tık · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>06 GSC - Organik Kanal · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>06 GSC - Organik Kanal · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
@@ -6568,7 +6568,7 @@
         </is>
       </c>
     </row>
-    <row r="165" ht="97.5" customHeight="1">
+    <row r="165" ht="111" customHeight="1">
       <c r="A165" s="5" t="inlineStr">
         <is>
           <t>https://www.banyoline.com</t>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E165" s="6" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="D200" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E200" s="6" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E201" s="6" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="D202" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E202" s="6" t="inlineStr">
@@ -8029,7 +8029,7 @@
       </c>
       <c r="D204" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
         </is>
       </c>
       <c r="E204" s="6" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E207" s="6" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E209" s="6" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="D210" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E210" s="6" t="inlineStr">
@@ -8288,7 +8288,7 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E211" s="6" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D212" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E212" s="6" t="inlineStr">
@@ -8362,7 +8362,7 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E213" s="6" t="inlineStr">
@@ -8399,7 +8399,7 @@
       </c>
       <c r="D214" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E214" s="6" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="D216" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E216" s="6" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="D218" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E218" s="6" t="inlineStr">
@@ -8621,7 +8621,7 @@
       </c>
       <c r="D220" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E220" s="6" t="inlineStr">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
@@ -8843,7 +8843,7 @@
       </c>
       <c r="D226" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E226" s="6" t="inlineStr">
@@ -8880,7 +8880,7 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E227" s="6" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="D230" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E230" s="6" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E231" s="6" t="inlineStr">
@@ -9065,7 +9065,7 @@
       </c>
       <c r="D232" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E232" s="6" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği · 28 Sonraki Adımlar</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="D234" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
@@ -9213,7 +9213,7 @@
       </c>
       <c r="D236" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
@@ -9250,7 +9250,7 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
@@ -9287,7 +9287,7 @@
       </c>
       <c r="D238" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="D240" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E240" s="6" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="E241" s="6" t="inlineStr">
@@ -50712,7 +50712,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -50837,7 +50837,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -50937,7 +50937,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -51037,7 +51037,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -51087,7 +51087,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -51162,7 +51162,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -51187,7 +51187,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -51312,7 +51312,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -51412,7 +51412,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -51437,7 +51437,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -51512,7 +51512,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -51562,7 +51562,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -51587,7 +51587,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -51687,7 +51687,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -51737,7 +51737,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -51787,7 +51787,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -51812,7 +51812,7 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -51837,7 +51837,7 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -51912,7 +51912,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -51987,7 +51987,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -52037,7 +52037,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -52062,7 +52062,7 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -52137,7 +52137,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -52162,7 +52162,7 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -52262,7 +52262,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -52287,7 +52287,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -52312,7 +52312,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -52413,7 +52413,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2.299 tekil kelime · Türkiye, Türkçe · aylık hacim Eyl 2022 - Ağu 2026 (talep grafiğinde Oca 2023 - Ağu 2026)</t>
+          <t>2.299 tekil kelime · Türkiye, Türkçe · aylık search volume Eyl 2022 - Ağu 2026 (talep grafiğinde Oca 2023 - Ağu 2026)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -52423,7 +52423,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Google Ads yakın yazım varyantlarına (çoğul, yazım farkı) aynı aylık seriyi döndürür; aynı seriye sahip kelimeler tek kelime olarak sayılmıştır (2.437 satırdan 2.349 tekil kelime); birleşen varyantlarda Türkçe ve yaygın yazım gösterilir (banyo batarya yerine banyo bataryası). Sezonsallık listesinde bulunmayan 19 kategori baş kelimesi (duşakabin, klozet fiyatları, tuvalet fırçası, musluk başlığı vb.) 04.10.2026 tarihinde eklenmiştir. Banyo Tezgahları altında yer alan ve banyo ya da lavabo içermeyen 21 mutfak ve genel tezgah araması (porselen tezgah, mermer tezgah, mutfak mermeri vb.) banyo mobilyası talebini yansıtmadığı için çıkarılmıştır. Kaynak listede banyo alt kategorisine eşlenmiş, ancak Google sonuçlarında banyo dışı ürünlere yönelen 25 genel ifade de (dolap kulpu ve salon konsolu, banyo ifadesi içermeyen çöp kovası, masa peçeteliği, elektronik panel, doğal taş traverten; 04.10.2026 kontrolü) ile marka adı geçen 4 arama evrenden çıkarılmıştır; marka aramaları Bölüm 09'da ayrıca ele alınmaktadır. Evren bu düzenlemelerle 2.299 kelimeye inmiştir. "lavabo" kelimesinde Keyword Planner Haziran 2025 - Mayıs 2026 arasında önceki ve sonraki aylardan 2-4 kat yüksek hacim göstermektedir; aynı dönemde Google Trends yalnızca yaklaşık %30'luk bir artış gösterdiği için bu aylar Trends seyrine göre yeniden ölçeklenmiştir. "wc" kelimesinin Haziran-Temmuz 2026 değerleri Dünya Kupası aramalarıyla karıştığı için 2025'in aynı aylarıyla değiştirilmiştir</t>
+          <t>Google Ads yakın yazım varyantlarına (çoğul, yazım farkı) aynı aylık seriyi döndürür; aynı seriye sahip kelimeler tek kelime olarak sayılmıştır (2.437 satırdan 2.349 tekil kelime); birleşen varyantlarda Türkçe ve yaygın yazım gösterilir (banyo batarya yerine banyo bataryası). Sezonsallık listesinde bulunmayan 19 kategori baş kelimesi (duşakabin, klozet fiyatları, tuvalet fırçası, musluk başlığı vb.) 04.10.2026 tarihinde eklenmiştir. Banyo Tezgahları altında yer alan ve banyo ya da lavabo içermeyen 21 mutfak ve genel tezgah araması (porselen tezgah, mermer tezgah, mutfak mermeri vb.) banyo mobilyası talebini yansıtmadığı için çıkarılmıştır. Kaynak listede banyo alt kategorisine eşlenmiş, ancak Google sonuçlarında banyo dışı ürünlere yönelen 25 genel ifade de (dolap kulpu ve salon konsolu, banyo ifadesi içermeyen çöp kovası, masa peçeteliği, elektronik panel, doğal taş traverten; 04.10.2026 kontrolü) ile marka adı geçen 4 arama evrenden çıkarılmıştır; marka aramaları Bölüm 09'da ayrıca ele alınmaktadır. Evren bu düzenlemelerle 2.299 kelimeye inmiştir. "lavabo" kelimesinde Keyword Planner Haziran 2025 - Mayıs 2026 arasında önceki ve sonraki aylardan 2-4 kat yüksek search volume göstermektedir; aynı dönemde Google Trends yalnızca yaklaşık %30'luk bir artış gösterdiği için bu aylar Trends seyrine göre yeniden ölçeklenmiştir. "wc" kelimesinin Haziran-Temmuz 2026 değerleri Dünya Kupası aramalarıyla karıştığı için 2025'in aynı aylarıyla değiştirilmiştir</t>
         </is>
       </c>
     </row>
@@ -52435,7 +52435,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>26 üretici marka ve 10 perakendeci · yalın marka adı ve marka + kategori aramaları · Türkiye, Türkçe · aylık hacim Eyl 2022 - Ağu 2026 · 04.10.2026</t>
+          <t>26 üretici marka ve 10 perakendeci · yalın marka adı ve marka + kategori aramaları · Türkiye, Türkçe · aylık search volume Eyl 2022 - Ağu 2026 · 04.10.2026</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -52445,7 +52445,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>"vitra" için kelime evrenindeki ifadelerin markalı biçimleri (2.227 ifade), rakipler için bunlardan VitrA'da hacmi olan 637 kategori ifadesi kullanılmıştır; yakın yazım varyantları marka ve kategori içinde tek sayılmış, " seramik" şirket adı araması olduğu için kategori hesabına alınmamıştır. "kale" kelimesi marka dışı anlamlar da taşır. Ahrefs'te rakip marka sitelerinin ve Trendyol, Hepsiburada, Koçtaş'ın sıralandığı marka ifadeleri (hacmi 10 ve üzeri, 04.10.2026) eklenmiştir; pazaryerlerinden yalnız banyo kategorisine eşlenen ifadeler, marka sitelerinden ayrıca servis, yedek parça ve satış noktası ifadeleri alınmış, ısıtma, kilit ve borsa gibi banyo dışı konular çıkarılmıştır. E.C.A. servis aramaları kombi servisinden ayrıştırılamadığı için alınmamıştır.</t>
+          <t>"vitra" için kelime evrenindeki ifadelerin markalı biçimleri (2.227 ifade), rakipler için bunlardan VitrA'da search volume olan 637 kategori ifadesi kullanılmıştır; yakın yazım varyantları marka ve kategori içinde tek sayılmış, " seramik" şirket adı araması olduğu için kategori hesabına alınmamıştır. "kale" kelimesi marka dışı anlamlar da taşır. Ahrefs'te rakip marka sitelerinin ve Trendyol, Hepsiburada, Koçtaş'ın sıralandığı marka ifadeleri (search volume 10 ve üzeri, 04.10.2026) eklenmiştir; pazaryerlerinden yalnız banyo kategorisine eşlenen ifadeler, marka sitelerinden ayrıca servis, yedek parça ve satış noktası ifadeleri alınmış, ısıtma, kilit ve borsa gibi banyo dışı konular çıkarılmıştır. E.C.A. servis aramaları kombi servisinden ayrıştırılamadığı için alınmamıştır.</t>
         </is>
       </c>
     </row>
@@ -52471,7 +52471,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="165" customHeight="1">
+    <row r="8" ht="178.5" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Google Analytics 4</t>
@@ -52489,7 +52489,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için oturum ve dönüşüm oranı Aralık öncesi ve sonrası kıyaslanmaz; gelir ve satın alma kıyaslanabilir. Giriş sayfası raporunda bir oturum birden fazla giriş sayfasında sayılabildiği için oturum pay olarak verilmiştir; gelir genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün geliri genel bakıştaki gelirden farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında oturum ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir. Sipariş onay sayfası keşiflerinde (1 Eki 2025 - 30 Eyl 2026) bazı aylar örneklendiği için yalnız paylar kullanılmış; satın almanın kaynak / ortamı GA4 atama modeline göre, oturum kanalı ise oturum kanal grubuna göre verilmiştir</t>
+          <t>Aralık 2025'te www.vitra.com.tr traffic'i aynı mülke katıldığı için session ve conversion rate Aralık öncesi ve sonrası kıyaslanmaz; revenue ve purchase kıyaslanabilir. Giriş sayfası raporunda bir session birden fazla giriş sayfasında sayılabildiği için session pay olarak verilmiştir; revenue genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün revenue'su genel bakıştaki revenue'dan farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında session ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir. Sipariş onay sayfası keşiflerinde (1 Eki 2025 - 30 Eyl 2026) bazı aylar örneklendiği için yalnız paylar kullanılmış; purchase'ın kaynak / ortamı GA4 atama modeline göre, session kanalı ise session kanal grubuna göre verilmiştir</t>
         </is>
       </c>
     </row>
@@ -52555,7 +52555,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Organik ve paid trafik değerleri Ahrefs tahminidir; gerçek ziyaret sayısı değildir</t>
+          <t>Organik ve paid traffic değerleri Ahrefs tahminidir; gerçek visit sayısı değildir</t>
         </is>
       </c>
     </row>
@@ -52691,7 +52691,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="57" customHeight="1">
+    <row r="18" ht="70.5" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Google arama sonuçları</t>
@@ -52699,7 +52699,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>322 kelime: A · VitrA gamı 159 (her alt kategoriden en az bir baş kelime), B · yakın kategori fırsatları 83, C · marka ve karşılaştırma 80; Keyword Planner'da hacmi olan · Türkiye, Türkçe, mobil · ilk 20 organik sonuç, AI Overview, PAA · 04.10.2026</t>
+          <t>322 kelime: A · VitrA gamı 159 (her alt kategoriden en az bir baş kelime), B · yakın kategori fırsatları 83, C · marka ve karşılaştırma 80; Keyword Planner'da search volume olan · Türkiye, Türkçe, mobil · ilk 20 organik sonuç, AI Overview, PAA · 04.10.2026</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -52731,7 +52731,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Yanıtlar kişiselleştirilmemiş oturumlardan alınmıştır ve aynı soruya gün içinde farklı yanıt verilebilir; oranlar yön göstericidir</t>
+          <t>Yanıtlar kişiselleştirilmemiş session'lardan alınmıştır ve aynı soruya gün içinde farklı yanıt verilebilir; oranlar yön göstericidir</t>
         </is>
       </c>
     </row>
@@ -52765,7 +52765,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>24 marka ve uzman site top pages ve 69 baş kelimenin sıralama verisi · Türkiye · 28.09.2026; bu bölümdeki arama hacimleri Google Keyword Planner (Eyl 2024 - Ağu 2026)</t>
+          <t>24 marka ve uzman site top pages ve 69 baş kelimenin sıralama verisi · Türkiye · 28.09.2026; bu bölümdeki search volume'ları Google Keyword Planner (Eyl 2024 - Ağu 2026)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -52797,7 +52797,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Kategori trafiği listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
+          <t>Kategori traffic'i listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
         </is>
       </c>
     </row>
@@ -52941,7 +52941,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Trendyol satıcı paneli: satış ve sipariş dağılımı (2025 Q4 - 2026 Q3), favori-görüntüleme (2025, 2026), 1.023 ürün ve 149 satıcı değerlendirmesi, 352 ürün sorusu, 44 Enleri listesi · Hepsiburada: hak ediş, görüntülenme, iptal, değerlendirme · 30.09.2026; ürün bazlı satış raporu, son 12 ay · 02.10.2026</t>
+          <t>Trendyol satıcı paneli: satış ve sipariş dağılımı (2025 Q4 - 2026 Q3), favori-görüntüleme (2025, 2026), 1.023 ürün ve 149 satıcı değerlendirmesi, 352 ürün sorusu, 44 Enleri listesi · Hepsiburada: hak ediş, view, iptal, değerlendirme · 30.09.2026; ürün bazlı satış raporu, son 12 ay · 02.10.2026</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -52951,7 +52951,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Yalnız resmi mağaza; ciro tutarı verilmez, pay ve oran kullanılır; temalar anahtar kelimeyle; Enleri ekran görüntüsünden okunmuştur</t>
+          <t>Yalnız resmi mağaza; revenue tutarı verilmez, pay ve oran kullanılır; temalar anahtar kelimeyle; Enleri ekran görüntüsünden okunmuştur</t>
         </is>
       </c>
     </row>
@@ -52973,7 +52973,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Rehber sayfaları adres yapısına göre konu gruplarına ayrılmıştır; en az 5 tık alan 93 sayfa değerlendirilmiştir</t>
+          <t>Rehber sayfaları adres yapısına göre konu gruplarına ayrılmıştır; en az 5 click alan 93 sayfa değerlendirilmiştir</t>
         </is>
       </c>
     </row>
@@ -53024,12 +53024,12 @@
     <row r="33" ht="43.5" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Similarweb site trafiği</t>
+          <t>Similarweb site traffic'i</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>31 alan adı: marka, uzman, yapı market, pazaryeri ve fiyat karşılaştırma siteleri; aylık ziyaret, kanal kırılımı, etkileşim · Haz - Ağu 2026 · 03.10.2026</t>
+          <t>31 alan adı: marka, uzman, yapı market, pazaryeri ve fiyat karşılaştırma siteleri; aylık visit, kanal kırılımı, etkileşim · Haz - Ağu 2026 · 03.10.2026</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -53039,7 +53039,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Ziyaretler tüm ülkeleri kapsayan tahminlerdir; aylık ziyareti ~35 binin altındaki 9 sitede kanal dağılımı modellendiği için gösterilmemiştir</t>
+          <t>Visit'ler tüm ülkeleri kapsayan tahminlerdir; aylık visit'i ~35 binin altındaki 9 sitede kanal dağılımı modellendiği için gösterilmemiştir</t>
         </is>
       </c>
     </row>
@@ -53083,7 +53083,7 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Click payı SEOmonitor'ün sıra ve hacimden türettiği tahmindir</t>
+          <t>Click payı SEOmonitor'ün sıra ve search volume'dan türettiği tahmindir</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trafik Türkçe; "Revenue'ya en çok katkı veren 15 ürün" tablosu tam genişlikte
- Metrik dönüşümünden trafik -> traffic kuralı kaldırıldı: başlık, içindekiler, sütun adları, metin, grafik verisi, Excel sekmeleri ve alt sayfalarda "trafik" (trafiği, trafikli, trafiğinin); Ahrefs "Traffic Potential" adı olduğu gibi
- Isı haritası sütun türü "trafiği" yazımını da tanıyor (renk imzası değişmedi)
- Resmi mağaza paneli: 15 ürün tablosu tam genişlikte, fiyat bandı grafiği ve tablosu altında yan yana

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -1517,7 +1517,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>06 GSC - Organik Kanal · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>06 GSC - Organik Kanal · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
@@ -6568,7 +6568,7 @@
         </is>
       </c>
     </row>
-    <row r="165" ht="111" customHeight="1">
+    <row r="165" ht="97.5" customHeight="1">
       <c r="A165" s="5" t="inlineStr">
         <is>
           <t>https://www.banyoline.com</t>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="E165" s="6" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="D200" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E200" s="6" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E201" s="6" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="D202" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E202" s="6" t="inlineStr">
@@ -8029,7 +8029,7 @@
       </c>
       <c r="D204" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
         </is>
       </c>
       <c r="E204" s="6" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E207" s="6" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E209" s="6" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="D210" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E210" s="6" t="inlineStr">
@@ -8288,7 +8288,7 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E211" s="6" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="D212" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E212" s="6" t="inlineStr">
@@ -8362,7 +8362,7 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E213" s="6" t="inlineStr">
@@ -8399,7 +8399,7 @@
       </c>
       <c r="D214" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E214" s="6" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="D216" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E216" s="6" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="D218" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="E218" s="6" t="inlineStr">
@@ -8621,7 +8621,7 @@
       </c>
       <c r="D220" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E220" s="6" t="inlineStr">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
@@ -8843,7 +8843,7 @@
       </c>
       <c r="D226" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E226" s="6" t="inlineStr">
@@ -8880,7 +8880,7 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E227" s="6" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="D230" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E230" s="6" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E231" s="6" t="inlineStr">
@@ -9065,7 +9065,7 @@
       </c>
       <c r="D232" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E232" s="6" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i · 28 Sonraki Adımlar</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="D234" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
@@ -9213,7 +9213,7 @@
       </c>
       <c r="D236" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
@@ -9250,7 +9250,7 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
@@ -9287,7 +9287,7 @@
       </c>
       <c r="D238" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="D240" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E240" s="6" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="E241" s="6" t="inlineStr">
@@ -50712,7 +50712,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -50837,7 +50837,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -50937,7 +50937,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
+          <t>14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -51037,7 +51037,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -51087,7 +51087,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -51162,7 +51162,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -51187,7 +51187,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -51312,7 +51312,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -51412,7 +51412,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -51437,7 +51437,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -51512,7 +51512,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -51562,7 +51562,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -51587,7 +51587,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -51687,7 +51687,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -51737,7 +51737,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -51787,7 +51787,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -51812,7 +51812,7 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -51837,7 +51837,7 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -51912,7 +51912,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -51987,7 +51987,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -52037,7 +52037,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -52062,7 +52062,7 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -52137,7 +52137,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -52162,7 +52162,7 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -52262,7 +52262,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -52287,7 +52287,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -52312,7 +52312,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Traffic'i</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -52489,7 +52489,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Aralık 2025'te www.vitra.com.tr traffic'i aynı mülke katıldığı için session ve conversion rate Aralık öncesi ve sonrası kıyaslanmaz; revenue ve purchase kıyaslanabilir. Giriş sayfası raporunda bir session birden fazla giriş sayfasında sayılabildiği için session pay olarak verilmiştir; revenue genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün revenue'su genel bakıştaki revenue'dan farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında session ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir. Sipariş onay sayfası keşiflerinde (1 Eki 2025 - 30 Eyl 2026) bazı aylar örneklendiği için yalnız paylar kullanılmış; purchase'ın kaynak / ortamı GA4 atama modeline göre, session kanalı ise session kanal grubuna göre verilmiştir</t>
+          <t>Aralık 2025'te www.vitra.com.tr trafiği aynı mülke katıldığı için session ve conversion rate Aralık öncesi ve sonrası kıyaslanmaz; revenue ve purchase kıyaslanabilir. Giriş sayfası raporunda bir session birden fazla giriş sayfasında sayılabildiği için session pay olarak verilmiştir; revenue genel bakışla birebir aynıdır. Anahtar olay (key event) satın alma dışında sepete ekleme, ödeme adımları, dosya indirme, favori ve üyelik olaylarını da kapsadığından kullanılmamıştır. Ürün raporunda sepete eklenen ürün (Items added to cart) beş ürün kodunda hatalı adet taşıdığı için bu kodlar, sepete ekleme olayının hatalı tetiklendiği Eylül 2026 ile birlikte oran hesabına katılmamış; ürün revenue'su genel bakıştaki revenue'dan farklı hesaplandığı için pay olarak verilmiştir. Sepet sayfasında session ve kullanıcı çerezi yenilendiği için kullanıcı düzeyindeki kırılımlar (yeni ve geri dönen kullanıcı, ilk kez satın alan) kullanılmamıştır. www.vitra.com.tr sayfaları (blog, koleksiyon, servis) bu mülkte Aralık 2025'ten itibaren ölçülmektedir. Sipariş onay sayfası keşiflerinde (1 Eki 2025 - 30 Eyl 2026) bazı aylar örneklendiği için yalnız paylar kullanılmış; purchase'ın kaynak / ortamı GA4 atama modeline göre, session kanalı ise session kanal grubuna göre verilmiştir</t>
         </is>
       </c>
     </row>
@@ -52555,7 +52555,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Organik ve paid traffic değerleri Ahrefs tahminidir; gerçek visit sayısı değildir</t>
+          <t>Organik ve paid trafik değerleri Ahrefs tahminidir; gerçek visit sayısı değildir</t>
         </is>
       </c>
     </row>
@@ -52797,7 +52797,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Kategori traffic'i listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
+          <t>Kategori trafiği listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
         </is>
       </c>
     </row>
@@ -53024,7 +53024,7 @@
     <row r="33" ht="43.5" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Similarweb site traffic'i</t>
+          <t>Similarweb site trafiği</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Bölüm 28 "Sonraki Adımlar İçin Öneriler": öncelik kademeleri kaldırıldı
- Öneri tablosunda Öncelik sütunu ve öncelik sıralaması yok; 34 öneri aksiyon, dayanak ve beklenen etkiyle veriliyor
- Giriş cümlesi: uygulama sırası VitrA ekibinin tercihleri, pazaryeri ve GA4 verisiyle birlikte belirlenebilir; "ilk adım olarak" üç maddelik kapanış içgörüsü kaldırıldı
- YouTube önerisindeki "(Bölüm 28, Öncelik 1)" atfı "(Bölüm 28)" oldu; Excel sekmesi "28.1 Sonraki Adım Önerileri"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -925,7 +925,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 28 Sonraki Adımlar</t>
+          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 14 Yeni Kategori ve Segment Fırsatları · 28 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 14 Yeni Kategori ve Segment Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 04 SSG ve BM: Derin Talep İncelemesi · 05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 GSC - Organik Kanal · 09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 04 SSG ve BM: Derin Talep İncelemesi · 05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 GSC - Organik Kanal · 09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>04 SSG ve BM: Derin Talep İncelemesi · 13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>04 SSG ve BM: Derin Talep İncelemesi · 13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 08 GA4 - Site ve E-Ticaret Performansı · 09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 11 YouTube: Montaj, Tamir ve Karar Videoları · 13 Katalog ve Talep Eşleşmesi · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>05 İhtiyaç Dili: Kullanıcı Ne Arıyor? · 06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 08 GA4 - Site ve E-Ticaret Performansı · 09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 11 YouTube: Montaj, Tamir ve Karar Videoları · 13 Katalog ve Talep Eşleşmesi · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>06 GSC - Organik Kanal · 07 Google Yapay Zeka Özellikleri ve Organik Click · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>09 Marka Aramaları ve Autocomplete · 10 Google Arama Sonuçları ve AI Overview · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 23 Kanal Politikaları ve Keşif Kanalları · 26 Kanal Rolleri ve Etkileşim Modeli · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>11 YouTube: Montaj, Tamir ve Karar Videoları · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>11 YouTube: Montaj, Tamir ve Karar Videoları · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>11 YouTube: Montaj, Tamir ve Karar Videoları · 28 Sonraki Adımlar</t>
+          <t>11 YouTube: Montaj, Tamir ve Karar Videoları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E131" s="6" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E141" s="6" t="inlineStr">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E161" s="6" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t>13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E162" s="6" t="inlineStr">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="D164" s="6" t="inlineStr">
         <is>
-          <t>13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar</t>
+          <t>13 Katalog ve Talep Eşleşmesi · 14 Yeni Kategori ve Segment Fırsatları · 15 Set, Komple Banyo ve Ürün + Hizmet · 26 Kanal Rolleri ve Etkileşim Modeli · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E164" s="6" t="inlineStr">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>14 Yeni Kategori ve Segment Fırsatları · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">
@@ -6901,7 +6901,7 @@
         </is>
       </c>
     </row>
-    <row r="174" ht="43.5" customHeight="1">
+    <row r="174" ht="57" customHeight="1">
       <c r="A174" s="5" t="inlineStr">
         <is>
           <t>https://www.bauhaus.info/service/leistungen/montageservice/komplettbad</t>
@@ -6919,7 +6919,7 @@
       </c>
       <c r="D174" s="6" t="inlineStr">
         <is>
-          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E174" s="6" t="inlineStr">
@@ -7197,7 +7197,7 @@
         </is>
       </c>
     </row>
-    <row r="182" ht="43.5" customHeight="1">
+    <row r="182" ht="57" customHeight="1">
       <c r="A182" s="5" t="inlineStr">
         <is>
           <t>https://www.koctas.com.tr/banyo-tadilati</t>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E182" s="6" t="inlineStr">
@@ -7271,7 +7271,7 @@
         </is>
       </c>
     </row>
-    <row r="184" ht="43.5" customHeight="1">
+    <row r="184" ht="57" customHeight="1">
       <c r="A184" s="5" t="inlineStr">
         <is>
           <t>https://reveal.kohler.com/en</t>
@@ -7289,7 +7289,7 @@
       </c>
       <c r="D184" s="6" t="inlineStr">
         <is>
-          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E184" s="6" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="D198" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E198" s="6" t="inlineStr">
@@ -8177,7 +8177,7 @@
       </c>
       <c r="D208" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E208" s="6" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği · 28 Sonraki Adımlar</t>
+          <t>17 Marka ve Uzman Sitelerde Kategori Trafiği · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="D309" s="6" t="inlineStr">
         <is>
-          <t>18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 28 Sonraki Adımlar</t>
+          <t>18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E309" s="6" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="D311" s="6" t="inlineStr">
         <is>
-          <t>18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E311" s="6" t="inlineStr">
@@ -15725,7 +15725,7 @@
       </c>
       <c r="D412" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E412" s="6" t="inlineStr">
@@ -20646,7 +20646,7 @@
       </c>
       <c r="D545" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E545" s="6" t="inlineStr">
@@ -26640,7 +26640,7 @@
       </c>
       <c r="D707" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E707" s="6" t="inlineStr">
@@ -32116,7 +32116,7 @@
       </c>
       <c r="D855" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E855" s="6" t="inlineStr">
@@ -35150,7 +35150,7 @@
       </c>
       <c r="D937" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E937" s="6" t="inlineStr">
@@ -39997,7 +39997,7 @@
       </c>
       <c r="D1068" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1068" s="6" t="inlineStr">
@@ -41255,7 +41255,7 @@
       </c>
       <c r="D1102" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1102" s="6" t="inlineStr">
@@ -41477,7 +41477,7 @@
       </c>
       <c r="D1108" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1108" s="6" t="inlineStr">
@@ -41810,7 +41810,7 @@
       </c>
       <c r="D1117" s="6" t="inlineStr">
         <is>
-          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar</t>
+          <t>19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1117" s="6" t="inlineStr">
@@ -42772,7 +42772,7 @@
       </c>
       <c r="D1143" s="6" t="inlineStr">
         <is>
-          <t>20 VitrA Resmi Mağaza: Pazaryeri Panel Verisi · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 28 Sonraki Adımlar</t>
+          <t>20 VitrA Resmi Mağaza: Pazaryeri Panel Verisi · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1143" s="6" t="inlineStr">
@@ -42809,7 +42809,7 @@
       </c>
       <c r="D1144" s="6" t="inlineStr">
         <is>
-          <t>20 VitrA Resmi Mağaza: Pazaryeri Panel Verisi · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 28 Sonraki Adımlar</t>
+          <t>20 VitrA Resmi Mağaza: Pazaryeri Panel Verisi · 21 Pazaryeri Yorumları ve Soru-Cevap: Sentiment ve Pain Point Analizi · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1144" s="6" t="inlineStr">
@@ -43013,7 +43013,7 @@
         </is>
       </c>
     </row>
-    <row r="1150" ht="43.5" customHeight="1">
+    <row r="1150" ht="57" customHeight="1">
       <c r="A1150" s="5" t="inlineStr">
         <is>
           <t>https://shopping.google.com</t>
@@ -43031,7 +43031,7 @@
       </c>
       <c r="D1150" s="6" t="inlineStr">
         <is>
-          <t>22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1150" s="6" t="inlineStr">
@@ -45214,7 +45214,7 @@
       </c>
       <c r="D1209" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1209" s="6" t="inlineStr">
@@ -45510,7 +45510,7 @@
       </c>
       <c r="D1217" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1217" s="6" t="inlineStr">
@@ -46287,7 +46287,7 @@
       </c>
       <c r="D1238" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1238" s="6" t="inlineStr">
@@ -46694,7 +46694,7 @@
       </c>
       <c r="D1249" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1249" s="6" t="inlineStr">
@@ -47212,7 +47212,7 @@
       </c>
       <c r="D1263" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1263" s="6" t="inlineStr">
@@ -47915,7 +47915,7 @@
       </c>
       <c r="D1282" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1282" s="6" t="inlineStr">
@@ -48063,7 +48063,7 @@
       </c>
       <c r="D1286" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1286" s="6" t="inlineStr">
@@ -48137,7 +48137,7 @@
       </c>
       <c r="D1288" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1288" s="6" t="inlineStr">
@@ -48359,7 +48359,7 @@
       </c>
       <c r="D1294" s="6" t="inlineStr">
         <is>
-          <t>24 vitra.com.tr Satın Alma Yolculuğu: Site İçi Arama, Sepet ve Ödeme · 28 Sonraki Adımlar</t>
+          <t>24 vitra.com.tr Satın Alma Yolculuğu: Site İçi Arama, Sepet ve Ödeme · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1294" s="6" t="inlineStr">
@@ -48396,7 +48396,7 @@
       </c>
       <c r="D1295" s="6" t="inlineStr">
         <is>
-          <t>24 vitra.com.tr Satın Alma Yolculuğu: Site İçi Arama, Sepet ve Ödeme · 28 Sonraki Adımlar</t>
+          <t>24 vitra.com.tr Satın Alma Yolculuğu: Site İçi Arama, Sepet ve Ödeme · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1295" s="6" t="inlineStr">
@@ -48415,7 +48415,7 @@
         </is>
       </c>
     </row>
-    <row r="1296" ht="30" customHeight="1">
+    <row r="1296" ht="43.5" customHeight="1">
       <c r="A1296" s="5" t="inlineStr">
         <is>
           <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
@@ -48433,7 +48433,7 @@
       </c>
       <c r="D1296" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1296" s="6" t="inlineStr">
@@ -48452,7 +48452,7 @@
         </is>
       </c>
     </row>
-    <row r="1297" ht="30" customHeight="1">
+    <row r="1297" ht="43.5" customHeight="1">
       <c r="A1297" s="5" t="inlineStr">
         <is>
           <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
@@ -48470,7 +48470,7 @@
       </c>
       <c r="D1297" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1297" s="6" t="inlineStr">
@@ -48489,7 +48489,7 @@
         </is>
       </c>
     </row>
-    <row r="1298" ht="30" customHeight="1">
+    <row r="1298" ht="43.5" customHeight="1">
       <c r="A1298" s="5" t="inlineStr">
         <is>
           <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
@@ -48507,7 +48507,7 @@
       </c>
       <c r="D1298" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1298" s="6" t="inlineStr">
@@ -48526,7 +48526,7 @@
         </is>
       </c>
     </row>
-    <row r="1299" ht="30" customHeight="1">
+    <row r="1299" ht="43.5" customHeight="1">
       <c r="A1299" s="5" t="inlineStr">
         <is>
           <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
@@ -48544,7 +48544,7 @@
       </c>
       <c r="D1299" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1299" s="6" t="inlineStr">
@@ -48600,7 +48600,7 @@
         </is>
       </c>
     </row>
-    <row r="1301" ht="30" customHeight="1">
+    <row r="1301" ht="43.5" customHeight="1">
       <c r="A1301" s="5" t="inlineStr">
         <is>
           <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
@@ -48618,7 +48618,7 @@
       </c>
       <c r="D1301" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1301" s="6" t="inlineStr">
@@ -48637,7 +48637,7 @@
         </is>
       </c>
     </row>
-    <row r="1302" ht="30" customHeight="1">
+    <row r="1302" ht="43.5" customHeight="1">
       <c r="A1302" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/banyonu-tasarla</t>
@@ -48655,7 +48655,7 @@
       </c>
       <c r="D1302" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1302" s="6" t="inlineStr">
@@ -48877,7 +48877,7 @@
       </c>
       <c r="D1308" s="6" t="inlineStr">
         <is>
-          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1308" s="6" t="inlineStr">
@@ -48914,7 +48914,7 @@
       </c>
       <c r="D1309" s="6" t="inlineStr">
         <is>
-          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1309" s="6" t="inlineStr">
@@ -48951,7 +48951,7 @@
       </c>
       <c r="D1310" s="6" t="inlineStr">
         <is>
-          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1310" s="6" t="inlineStr">
@@ -48988,7 +48988,7 @@
       </c>
       <c r="D1311" s="6" t="inlineStr">
         <is>
-          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="E1311" s="6" t="inlineStr">
@@ -50462,7 +50462,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>12 Şikayetvar: Satış Sonrası Deneyim · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>12 Şikayetvar: Satış Sonrası Deneyim · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -50587,7 +50587,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>11 YouTube: Montaj, Tamir ve Karar Videoları · 23 Kanal Politikaları ve Keşif Kanalları · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>11 YouTube: Montaj, Tamir ve Karar Videoları · 23 Kanal Politikaları ve Keşif Kanalları · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -50612,7 +50612,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -50637,7 +50637,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>16 Rakip Görünürlüğü ve Kanal Ölçeği · 18 Pazaryerleri: Kategori Yapısı ve Çok Satanlar · 19 Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · 22 Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -50912,7 +50912,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 28 Sonraki Adımlar</t>
+          <t>02 Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -51112,7 +51112,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>23 Kanal Politikaları ve Keşif Kanalları · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -51262,7 +51262,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -51287,7 +51287,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -51387,7 +51387,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -51487,7 +51487,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -51637,7 +51637,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -51662,7 +51662,7 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>03 Kategori Talebi ve Dönemsel Değişim · 14 Yeni Kategori ve Segment Fırsatları · 28 Sonraki Adımlar</t>
+          <t>03 Kategori Talebi ve Dönemsel Değişim · 14 Yeni Kategori ve Segment Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -51712,7 +51712,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -51862,7 +51862,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>15 Set, Komple Banyo ve Ürün + Hizmet · 25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -51987,7 +51987,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar</t>
+          <t>10 Google Arama Sonuçları ve AI Overview · 16 Rakip Görünürlüğü ve Kanal Ölçeği · 17 Marka ve Uzman Sitelerde Kategori Trafiği · 27 AI Arama ve GEO Fırsatları · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -52187,7 +52187,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar</t>
+          <t>25 Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · 28 Sonraki Adımlar İçin Öneriler</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Marka revizeleri: Banyomu Yenilemek İstiyorum formu kaldırıldı, taksit yorumları 9 vade farksız / 12 vade farklı ayrımına göre güncellendi; Partial rozeti çevirisi düzeltildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
+++ b/VitrA_E-Ticaret_Kaynak_Siteler.xlsx
@@ -1536,7 +1536,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="124.5" customHeight="1">
+    <row r="29" ht="84" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr</t>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>VitrA ana sayfa: şerit mesajları ve Banyo Asistanı akışı (taksit, kargo ve hizmet mesajı) | Rakip görünürlüğü ve kanal ölçeği: vitra.com.tr alan adı metrikleri (Ahrefs, Türkiye) | Marka ve uzman sitelerde kategori trafiği: vitra.com.tr tema × trafik matrisi (Ahrefs, Türkiye) | vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (ana sayfa)</t>
+          <t>VitrA ana sayfa: şerit mesajları (taksit ve kargo) | Rakip görünürlüğü ve kanal ölçeği: vitra.com.tr alan adı metrikleri (Ahrefs, Türkiye) | Marka ve uzman sitelerde kategori trafiği: vitra.com.tr tema × trafik matrisi (Ahrefs, Türkiye) | vitra.com.tr organik kanal performansı: sayfa bazında tıklama ve gösterim (ana sayfa)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1559,12 +1559,12 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Şeritte 'tüm ürünlerde vade farksız 6 ay taksit' ve 'tüm ürünlerde ücretsiz kargo'; Banyo Asistanı (Banyomu Yenilemek İstiyorum) 4 adımlı lead akışı: telefon, mağaza veya görüntülü görüşme seçimi, slot, WhatsApp teyidi; %40'a varan indirim, 9 taksit, ücretsiz mimari projelendirme | Batch Analysis: DR 66, 7.428 organik kelime, ilk 3'te 4.127 kelime, 330.499 organik ve 50.286 paid trafik (Ahrefs tahmini, 27.09.2026) | Ahrefs site toplamı: DR 66, 7.428 organik kelime, 330.499 aylık organik trafik; top pages: 138 sayfa 40'tan fazla temaya eşlendi (28.09.2026) | 1 Eki 2025 - 30 Eyl 2026: 134.587 tıklama, 4.500.313 gösterim, ortalama sıra 10</t>
+          <t>Şeritte 'tüm ürünlerde vade farksız 9 ay taksit' ve 'tüm ürünlerde ücretsiz kargo' | Batch Analysis: DR 66, 7.428 organik kelime, ilk 3'te 4.127 kelime, 330.499 organik ve 50.286 paid trafik (Ahrefs tahmini, 27.09.2026) | Ahrefs site toplamı: DR 66, 7.428 organik kelime, 330.499 aylık organik trafik; top pages: 138 sayfa 40'tan fazla temaya eşlendi (28.09.2026) | 1 Eki 2025 - 30 Eyl 2026: 134.587 tıklama, 4.500.313 gösterim, ortalama sıra 10</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>27.09.2026 · 28.09.2026 · 29.09.2026</t>
+          <t>27.09.2026 · 28.09.2026 · 10.10.2026</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -47883,7 +47883,7 @@
       </c>
       <c r="E1281" s="6" t="inlineStr">
         <is>
-          <t>Ürün tablosunda 12 taksite kadar seçenek (8, 9 ve 12 taksit çoğu kartta vade farklı, 2-3-4-6 taksit eşit tutar); tahmini kargoya teslim tarihi; 30 güne kadar ücretsiz iade ifadesi; montaj hizmeti seçeneği (+₺5.300)</t>
+          <t>Ürün tablosunda vade farkıyla 12 taksite kadar seçenek; tahmini kargoya teslim tarihi; 30 güne kadar ücretsiz iade ifadesi; montaj hizmeti seçeneği (+₺5.300)</t>
         </is>
       </c>
       <c r="F1281" s="7" t="inlineStr">
@@ -50551,7 +50551,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="43.5" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>vitra.com.tr</t>
@@ -50572,7 +50572,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>27.09.2026 · 28.09.2026 · 29.09.2026 · 30.09.2026 · 02.10.2026 · 04.10.2026</t>
+          <t>27.09.2026 · 28.09.2026 · 29.09.2026 · 30.09.2026 · 02.10.2026 · 04.10.2026 · 10.10.2026</t>
         </is>
       </c>
     </row>
@@ -52589,7 +52589,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>7.804 ürün adresi · hizmet, kategori ve ürün sayfaları · Banyo Asistanı · 28.09.2026</t>
+          <t>7.804 ürün adresi · hizmet, kategori ve ürün sayfaları · 28.09.2026</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">

</xml_diff>